<commit_message>
Add occupation breakdown, author-controlled altitude, and generic footer
- demo_data.xlsx: new Occupation column (scoreboard range grown to D3:G9),
  values seeded-random from {Tech Arch, Developer, DM};
  scripts/add_occupation.py regenerates it reproducibly.
- levels.html: 'By occupation' totals in the Executive view, Occupation in
  the Summary column and detail facts, and a source-agnostic footer.
- Author-controlled opening altitude via an optional 'detail' parameter;
  scripts/make_levels_sample.py builds levels_sample.xlsx to demonstrate it.
- Rendered-output checks updated/added (test_levels_render.py,
  test_levels_author.py).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo_data.xlsx
+++ b/demo_data.xlsx
@@ -1,115 +1,50 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="Parameters">Sheet1!$A$3:$B$5</definedName>
-    <definedName name="scoreboard">Sheet1!$D$3:$F$9</definedName>
+    <definedName name="scoreboard">Sheet1!$D$3:$G$9</definedName>
   </definedNames>
-  <calcPr/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>Tables Demo</t>
-  </si>
-  <si>
-    <t>First Name</t>
-  </si>
-  <si>
-    <t>Last Name</t>
-  </si>
-  <si>
-    <t>Points</t>
-  </si>
-  <si>
-    <t>version</t>
-  </si>
-  <si>
-    <t>0.1.2</t>
-  </si>
-  <si>
-    <t>Jill</t>
-  </si>
-  <si>
-    <t>Smith</t>
-  </si>
-  <si>
-    <t>board_data</t>
-  </si>
-  <si>
-    <t>[scoreboard]</t>
-  </si>
-  <si>
-    <t>Eve</t>
-  </si>
-  <si>
-    <t>Jackson</t>
-  </si>
-  <si>
-    <t>Adam</t>
-  </si>
-  <si>
-    <t>Johnson</t>
-  </si>
-  <si>
-    <t>Steve</t>
-  </si>
-  <si>
-    <t>Holden</t>
-  </si>
-  <si>
-    <t>Steven</t>
-  </si>
-  <si>
-    <t>Pugh</t>
-  </si>
-  <si>
-    <t>John</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="4">
     <font>
-      <sz val="10.0"/>
+      <name val="Arial"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <sz val="10"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Arial"/>
       <color theme="1"/>
-      <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11.0"/>
+      <name val="Verdana"/>
+      <b val="1"/>
       <color rgb="FF000000"/>
-      <name val="Verdana"/>
+      <sz val="11"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <name val="Verdana"/>
       <color rgb="FF000000"/>
-      <name val="Verdana"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
@@ -125,34 +60,93 @@
     <border/>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" vertical="top"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -350,111 +344,190 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:G9"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1"/>
+      <c r="A1" s="1" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>4</v>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Tables Demo</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>First Name</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Last Name</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Occupation</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="4">
-        <v>50.0</v>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>0.1.2</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Jill</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Smith</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="4">
-        <v>94.0</v>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>board_data</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>[scoreboard]</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Eve</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>94</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Tech Arch</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="D6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="4">
-        <v>67.0</v>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Adam</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Johnson</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="D7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" s="4">
-        <v>67.0</v>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Steve</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Holden</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Tech Arch</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="D8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="4">
-        <v>98.0</v>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Steven</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Pugh</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>98</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Tech Arch</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="D9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" s="4">
-        <v>123.0</v>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>John</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Johnson</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>123</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Nest version into a {number} dict; render version.number
version is now a one-row {version} named range (number | 0.1.2), relying on
the hubris flatten fix so a single-entry dict is not flattened to a vector.
scripts/nest_version.py regenerates it; levels_sample.xlsx refreshed. All four
templates render version.number.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo_data.xlsx
+++ b/demo_data.xlsx
@@ -8,6 +8,7 @@
   <definedNames>
     <definedName name="Parameters">Sheet1!$A$3:$B$5</definedName>
     <definedName name="scoreboard">Sheet1!$D$3:$G$9</definedName>
+    <definedName name="version">Sheet1!$A$11:$B$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -349,7 +350,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
@@ -381,7 +382,7 @@
           <t>Points</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="0" t="inlineStr">
         <is>
           <t>Occupation</t>
         </is>
@@ -395,7 +396,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>0.1.2</t>
+          <t>{version}</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -411,7 +412,7 @@
       <c r="F4" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="0" t="inlineStr">
         <is>
           <t>DM</t>
         </is>
@@ -441,7 +442,7 @@
       <c r="F5" s="4" t="n">
         <v>94</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="0" t="inlineStr">
         <is>
           <t>Tech Arch</t>
         </is>
@@ -461,7 +462,7 @@
       <c r="F6" s="4" t="n">
         <v>67</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" s="0" t="inlineStr">
         <is>
           <t>Developer</t>
         </is>
@@ -481,7 +482,7 @@
       <c r="F7" s="4" t="n">
         <v>67</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="0" t="inlineStr">
         <is>
           <t>Tech Arch</t>
         </is>
@@ -501,7 +502,7 @@
       <c r="F8" s="4" t="n">
         <v>98</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" s="0" t="inlineStr">
         <is>
           <t>Tech Arch</t>
         </is>
@@ -521,9 +522,21 @@
       <c r="F9" s="4" t="n">
         <v>123</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" s="0" t="inlineStr">
         <is>
           <t>Developer</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0.1.2</t>
         </is>
       </c>
     </row>

</xml_diff>